<commit_message>
the final projectt update_thanks for everything
</commit_message>
<xml_diff>
--- a/orange_part/emails_output/emails.xlsx
+++ b/orange_part/emails_output/emails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>UID</t>
   </si>
@@ -25,7 +25,10 @@
     <t>Attachments</t>
   </si>
   <si>
-    <t>31</t>
+    <t>39</t>
+  </si>
+  <si>
+    <t>40</t>
   </si>
   <si>
     <t>Yessine Ht &lt;yessineht@gmail.com&gt;
@@ -95,27 +98,264 @@
     <t>From: /*MailSender*/Yessine Ht &lt;yessineht@gmail.com&gt;/*MailSender*/ 
  Subject: /*MailSub*/Mission Order Request/*MailSub*/ 
  Date: Tue, 19 May 2026 21:42:45 +0100 
- J'espère que vous allez bien ! Je me permets de vous contacter afin de_x000D_
-solliciter votre validation pour un court déplacement professionnel prévu_x000D_
-les 17 et 18 novembre 2024 à Kairouan. Cette mission est liée à des_x000D_
-activités en cours qui nécessitent vraiment une présence sur place, et je_x000D_
-souhaite m'assurer que tout se passe dans les meilleures conditions._x000D_
-_x000D_
-Voici mes informations pour la demande : je m'appelle Imen Souissi, vous_x000D_
-pouvez me joindre à l'adresse yessineht@gmail.com, et la destination est_x000D_
-Kairouan pour ces deux journées. L'accord de mon responsable est encore en_x000D_
-attente, mais je souhaitais vous transmettre cette demande en avance afin_x000D_
-d'éviter tout délai de traitement._x000D_
-_x000D_
-Si vous avez besoin de quoi que ce soit de ma part — documents_x000D_
-supplémentaires, détails sur les objectifs de la mission, ou autre —_x000D_
-n'hésitez pas à me le faire savoir et je vous fournirai tout cela dans les_x000D_
-plus brefs délais._x000D_
-_x000D_
-Merci beaucoup pour votre aide et votre disponibilité !_x000D_
+ J'espère que vous allez bien ! Je me permets de vous contacter afin de_x005F_x000D_
+solliciter votre validation pour un court déplacement professionnel prévu_x005F_x000D_
+les 17 et 18 novembre 2024 à Kairouan. Cette mission est liée à des_x005F_x000D_
+activités en cours qui nécessitent vraiment une présence sur place, et je_x005F_x000D_
+souhaite m'assurer que tout se passe dans les meilleures conditions._x005F_x000D_
+_x005F_x000D_
+Voici mes informations pour la demande : je m'appelle Imen Souissi, vous_x005F_x000D_
+pouvez me joindre à l'adresse yessineht@gmail.com, et la destination est_x005F_x000D_
+Kairouan pour ces deux journées. L'accord de mon responsable est encore en_x005F_x000D_
+attente, mais je souhaitais vous transmettre cette demande en avance afin_x005F_x000D_
+d'éviter tout délai de traitement._x005F_x000D_
+_x005F_x000D_
+Si vous avez besoin de quoi que ce soit de ma part — documents_x005F_x000D_
+supplémentaires, détails sur les objectifs de la mission, ou autre —_x005F_x000D_
+n'hésitez pas à me le faire savoir et je vous fournirai tout cela dans les_x005F_x000D_
+plus brefs délais._x005F_x000D_
+_x005F_x000D_
+Merci beaucoup pour votre aide et votre disponibilité !_x005F_x000D_
+_x005F_x000D_
+Cordialement,_x005F_x000D_
+yessine haj taieb</t>
+  </si>
+  <si>
+    <t>From: /*MailSender*/Yessine Ht &lt;yessineht@gmail.com&gt;/*MailSender*/ 
+ Subject: /*MailSub*/Demande de recrutement – Poste : Développeur Full Stack/*MailSub*/ 
+ Date: Thu, 21 May 2026 09:45:19 +0100 
+ Madame, Monsieur,_x005F_x000D_
+_x005F_x000D_
+Je me permets de vous adresser la présente afin d'initier une demande de_x005F_x000D_
+recrutement pour le poste de Développeur Full Stack au sein de notre_x005F_x000D_
+département Informatique._x005F_x000D_
+_x005F_x000D_
+**Description du besoin**_x005F_x000D_
+Face à l'accroissement de nos projets de développement, nous avons besoin_x005F_x000D_
+de renforcer notre équipe technique par le recrutement d'un profil_x005F_x000D_
+expérimenté en développement web Full Stack._x005F_x000D_
+_x005F_x000D_
+**Poste**_x005F_x000D_
+Développeur Full Stack_x005F_x000D_
+_x005F_x000D_
+**Documents joints**_x005F_x000D_
+- Fiche de poste : ci-jointe_x005F_x000D_
+- Questionnaire de recrutement : ci-joint_x005F_x000D_
+_x005F_x000D_
+**Présélection des candidats**_x005F_x000D_
+Suite à l'analyse des candidatures reçues, les candidats présélectionnés_x005F_x000D_
+sont les suivants :_x005F_x000D_
+1. Ahmed Ben Salem_x005F_x000D_
+2. Sonia Trabelsi_x005F_x000D_
+3. Karim Mansour_x005F_x000D_
+_x005F_x000D_
+**Entretien(s)**_x005F_x000D_
+- Date d'entretien : 28/05/2026_x005F_x000D_
+- Type d'entretien : Entretien technique + RH_x005F_x000D_
+- Évaluateurs : M. Youssef Chaabane (Responsable technique), Mme Rim_x005F_x000D_
+Bouaziz (RH)_x005F_x000D_
+_x005F_x000D_
+**Résultats**_x005F_x000D_
+- Résultats des questionnaires : ci-joints_x005F_x000D_
+- Résultat de l'entretien : Favorable pour M. Ahmed Ben Salem_x005F_x000D_
+_x005F_x000D_
+**Candidat retenu**_x005F_x000D_
+- Nom du candidat retenu : Ahmed Ben Salem_x005F_x000D_
+- Type de contrat : CDI_x005F_x000D_
+- Date d'embauche : 01/07/2026_x005F_x000D_
+- Seuil de proposition d'embauche : 2 800 TND_x005F_x000D_
+- Proposition finale d'embauche : 3 000 TND_x005F_x000D_
+_x005F_x000D_
+Nous vous prions de bien vouloir procéder à la préparation du contrat et de_x005F_x000D_
+planifier la signature dans les meilleurs délais._x005F_x000D_
+_x005F_x000D_
+Contrat : à établir_x005F_x000D_
+_x005F_x000D_
+Restant à votre disposition pour tout complément d'information,_x005F_x000D_
+_x005F_x000D_
+Cordialement,_x005F_x000D_
+_x005F_x000D_
+Mohamed Khalil_x005F_x000D_
+Responsable Département Informatique_x005F_x000D_
+m.khalil@entreprise.tn | +216 71 000 000</t>
+  </si>
+  <si>
+    <t>From: /*MailSender*/Yessine Ht &lt;yessineht@gmail.com&gt;/*MailSender*/ 
+ Subject: /*MailSub*/Évaluation de fin de période d'essai – Mme Sonia Trabelsi/*MailSub*/ 
+ Date: Thu, 21 May 2026 09:48:26 +0100 
+ Madame, Monsieur,_x005F_x000D_
+_x005F_x000D_
+Je vous transmets ci-dessous le rapport d'évaluation de fin de période_x005F_x000D_
+d'essai concernant Mme Sonia Trabelsi, intégrée au sein du département_x005F_x000D_
+Ressources Humaines depuis le 01/03/2026._x005F_x000D_
+_x005F_x000D_
+━━━━━━━━━━━━━━━━━━━━━━━━_x005F_x000D_
+I. ÉVALUATION PAR LE SUPÉRIEUR HIÉRARCHIQUE_x005F_x000D_
+━━━━━━━━━━━━━━━━━━━━━━━━_x005F_x000D_
+_x005F_x000D_
+Collaborateur évalué : Mme Sonia Trabelsi_x005F_x000D_
+Responsable évaluateur : M. Youssef Chaabane – Responsable RH_x005F_x000D_
+_x005F_x000D_
+• Connaissance de l'emploi : Bonne maîtrise des procédures internes et des_x005F_x000D_
+outils RH utilisés. S'est rapidement approprié les processus en place._x005F_x000D_
+_x005F_x000D_
+• Productivité (Qualité / Quantité de travail) : Travail soigné et livré_x005F_x000D_
+dans les délais impartis. Volume de tâches traitées conforme aux attentes_x005F_x000D_
+du poste._x005F_x000D_
+_x005F_x000D_
+• Fiabilité : Ponctuelle, rigoureuse et respectueuse de ses engagements._x005F_x000D_
+Aucune absence non justifiée durant la période d'essai._x005F_x000D_
+_x005F_x000D_
+• Collaboration : S'intègre facilement dans les dynamiques d'équipe._x005F_x000D_
+Participe activement aux réunions et contribue aux projets collectifs._x005F_x000D_
+_x005F_x000D_
+• Adaptabilité : A démontré une bonne capacité d'adaptation face aux_x005F_x000D_
+changements de priorités et aux situations imprévues._x005F_x000D_
+_x005F_x000D_
+• Initiative : Fait preuve d'empressement et de proactivité. A proposé_x005F_x000D_
+plusieurs améliorations sur les procédures de suivi des candidatures._x005F_x000D_
+_x005F_x000D_
+• Service à la clientèle / fournisseurs : Interactions professionnelles et_x005F_x000D_
+courtoises avec les partenaires externes et les candidats._x005F_x000D_
+_x005F_x000D_
+• Commentaire général : Mme Trabelsi est une collaboratrice sérieuse et_x005F_x000D_
+investie. Son intégration au sein de l'équipe s'est déroulée de manière_x005F_x000D_
+très satisfaisante._x005F_x000D_
+_x005F_x000D_
+━━━━━━━━━━━━━━━━━━━━━━━━_x005F_x000D_
+II. ÉVALUATION RH_x005F_x000D_
+━━━━━━━━━━━━━━━━━━━━━━━━_x005F_x000D_
+_x005F_x000D_
+• Attitudes et comportements au travail : Comportement exemplaire,_x005F_x000D_
+respectueux des valeurs et du règlement intérieur de l'entreprise._x005F_x000D_
+_x005F_x000D_
+• Motivation et satisfaction personnelle : Se déclare motivée par ses_x005F_x000D_
+missions et exprime un intérêt marqué pour évoluer au sein du département._x005F_x000D_
+_x005F_x000D_
+• Environnement de travail et organisation générale : S'est bien adaptée à_x005F_x000D_
+l'environnement de travail. Espace de travail organisé, gestion du temps_x005F_x000D_
+satisfaisante._x005F_x000D_
+_x005F_x000D_
+• Encadrement et intégration : L'accompagnement réalisé durant la période_x005F_x000D_
+d'essai a été jugé suffisant. La collaboratrice a bénéficié d'un suivi_x005F_x000D_
+régulier par son responsable direct._x005F_x000D_
+_x005F_x000D_
+• Écarts constatés : Légère marge de progression identifiée sur la gestion_x005F_x000D_
+des priorités en période de forte charge. Point à suivre lors du prochain_x005F_x000D_
+entretien annuel._x005F_x000D_
+_x005F_x000D_
+• Relation avec les collègues au sein du département : Excellentes_x005F_x000D_
+relations interpersonnelles. Appréciée par l'ensemble de l'équipe pour son_x005F_x000D_
+esprit d'entraide._x005F_x000D_
+_x005F_x000D_
+• Ambition exprimée : Souhaite à terme prendre en charge le volet formation_x005F_x000D_
+et développement des compétences au sein du département RH._x005F_x000D_
+_x005F_x000D_
+• Proposition d'amélioration : Nous recommandons de lui confier_x005F_x000D_
+progressivement des missions de coordination afin de développer ses_x005F_x000D_
+compétences managériales._x005F_x000D_
+_x005F_x000D_
+━━━━━━━━━━━━━━━━━━━━━━━━_x005F_x000D_
+III. DÉCISION_x005F_x000D_
+━━━━━━━━━━━━━━━━━━━━━━━━_x005F_x000D_
+_x005F_x000D_
+• Décision proposée : Confirmation de la titularisation à l'issue de la_x005F_x000D_
+période d'essai._x005F_x000D_
+• Décision finale : FAVORABLE – Intégration définitive au sein du_x005F_x000D_
+département RH à compter du 01/06/2026._x005F_x000D_
+_x005F_x000D_
+Nous vous prions de bien vouloir prendre note de cette décision et de_x005F_x000D_
+procéder aux formalités administratives nécessaires à la confirmation du_x005F_x000D_
+contrat._x005F_x000D_
+_x005F_x000D_
+Restant à votre disposition pour tout complément d'information,_x005F_x000D_
+_x005F_x000D_
+Cordialement,_x005F_x000D_
+_x005F_x000D_
+Mme Rim Bouaziz_x005F_x000D_
+Chargée des Ressources Humaines_x005F_x000D_
+r.bouaziz@entreprise.tn | +216 71 000 001</t>
+  </si>
+  <si>
+    <t>From: /*MailSender*/Yessine Ht &lt;yessineht@gmail.com&gt;/*MailSender*/ 
+ Subject: /*MailSub*/Demande d'autorisation d'absence – 27/05/2026/*MailSub*/ 
+ Date: Thu, 21 May 2026 11:27:18 +0100 
+ Madame, Monsieur,_x005F_x000D_
+_x005F_x000D_
+Je me permets de vous adresser la présente afin de solliciter une_x005F_x000D_
+autorisation d'absence pour des raisons personnelles._x005F_x000D_
+_x005F_x000D_
+• Type d'autorisation : Autorisation de sortie exceptionnelle_x005F_x000D_
+• Date de l'absence : 27/05/2026_x005F_x000D_
+• Heure de départ : 10h00_x005F_x000D_
+• Heure de retour : 13h30_x005F_x000D_
+• Nombre d'heures : 3h30_x005F_x000D_
+• Motif de l'absence : Rendez-vous médical spécialisé ne pouvant être_x005F_x000D_
+reporté_x005F_x000D_
+_x005F_x000D_
+Je m'engage à assurer la continuité de mes tâches en amont et à rattraper_x005F_x000D_
+le temps d'absence si cela s'avère nécessaire._x005F_x000D_
+_x005F_x000D_
+Dans l'attente de votre accord, je reste disponible pour tout échange à ce_x005F_x000D_
+sujet._x005F_x000D_
+_x005F_x000D_
+Cordialement,_x005F_x000D_
+_x005F_x000D_
+Ahmed Ben Salem_x005F_x000D_
+Développeur Full Stack – Département Informatique_x005F_x000D_
+a.bensalem@entreprise.tn | +216 55 000 123</t>
+  </si>
+  <si>
+    <t>From: /*MailSender*/Rayen gargouri &lt;gargourirayen@gmail.com&gt;/*MailSender*/ 
+ Subject: /*MailSub*/Demande d'activation d'une offre Fibre Entreprise/*MailSub*/ 
+ Date: Wed, 3 Jun 2026 00:28:44 +0100 
+ Bonjour,_x000D_
+_x000D_
+Je représente la société TechSolutions et nous souhaitons souscrire à une_x000D_
+offre Fibre Entreprise pour notre nouveau siège situé à Sfax._x000D_
+_x000D_
+Avant de finaliser notre choix, nous aimerions obtenir des informations_x000D_
+concernant les débits disponibles, les délais d'installation, les garanties_x000D_
+de disponibilité du service ainsi que les tarifs applicables aux_x000D_
+entreprises._x000D_
+_x000D_
+Pourriez-vous également nous indiquer les documents nécessaires à la_x000D_
+souscription et les coordonnées d'un conseiller commercial pouvant nous_x000D_
+accompagner dans cette démarche ?_x000D_
+_x000D_
+Je vous remercie pour votre aide et reste dans l'attente de votre retour._x000D_
 _x000D_
 Cordialement,_x000D_
-yessine haj taieb</t>
+_x000D_
+Mohamed Rayen GARGOURI_x000D_
+Responsable Administratif</t>
+  </si>
+  <si>
+    <t>From: /*MailSender*/Rayen gargouri &lt;gargourirayen@gmail.com&gt;/*MailSender*/ 
+ Subject: /*MailSub*/Réclamation concernant des coupures répétées de la connexion Internet/*MailSub*/ 
+ Date: Wed, 3 Jun 2026 00:30:12 +0100 
+ Bonjour,_x000D_
+_x000D_
+Je me permets de vous contacter afin de signaler un problème récurrent_x000D_
+affectant ma connexion Internet Orange._x000D_
+_x000D_
+Depuis environ une semaine, je constate plusieurs coupures quotidiennes qui_x000D_
+interrompent régulièrement mes activités professionnelles en télétravail._x000D_
+Malgré plusieurs redémarrages du routeur, le problème persiste et la_x000D_
+qualité de la connexion reste très instable._x000D_
+_x000D_
+Cette situation me cause un réel préjudice et je souhaiterais qu'une_x000D_
+vérification technique soit effectuée dans les meilleurs délais afin_x000D_
+d'identifier l'origine du dysfonctionnement._x000D_
+_x000D_
+Je vous remercie de bien vouloir prendre en compte ma réclamation et de me_x000D_
+tenir informé des actions entreprises._x000D_
+_x000D_
+Cordialement,_x000D_
+_x000D_
+Mohamed Rayen GARGOURI_x000D_
+Client_x000D_
+Numéro de ligne : 52 123 456</t>
   </si>
   <si>
     <t>Doctor_Note_with_Signature.pdf</t>
@@ -456,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -475,7 +715,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -483,10 +723,10 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -494,10 +734,10 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -505,18 +745,58 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
-        <v>8</v>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>